<commit_message>
Mise à jours prestations
</commit_message>
<xml_diff>
--- a/input.xlsx
+++ b/input.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/25a393584c41f6f2/Documents/Mon Patrimoine/Projet Immobilier/2023 Terrasses de Galieni/09 - Copropriété/Site de calcul des charges de copropriété/streamlit-copro-charges/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1352" documentId="13_ncr:1_{471232EB-3AAB-4D08-BC1C-7B7CD1C1D853}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ABBA670F-8EBD-46A0-88D7-23996C8CEBB2}"/>
+  <xr:revisionPtr revIDLastSave="1365" documentId="13_ncr:1_{471232EB-3AAB-4D08-BC1C-7B7CD1C1D853}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EA551C85-FA08-408F-B843-E797C6AF88DC}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="593" uniqueCount="405">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="599" uniqueCount="408">
   <si>
     <t>Taxes</t>
   </si>
@@ -1268,6 +1268,15 @@
   </si>
   <si>
     <t>Prix TTC de l'unité</t>
+  </si>
+  <si>
+    <t>Contrat d'entretien de la chaudière à gaz, bois et granules Dalkia</t>
+  </si>
+  <si>
+    <t>Dalkia</t>
+  </si>
+  <si>
+    <t>Contrat P2, engagement sur 3 ans, a priori pas de livraison</t>
   </si>
 </sst>
 </file>
@@ -1367,16 +1376,7 @@
   </cellStyles>
   <dxfs count="31">
     <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$€-40C]_-;\-* #,##0.00\ [$€-40C]_-;_-* &quot;-&quot;??\ [$€-40C]_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <font>
@@ -1395,16 +1395,61 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
-      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$€-40C]_-;\-* #,##0.00\ [$€-40C]_-;_-* &quot;-&quot;??\ [$€-40C]_-;_-@_-"/>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
     </dxf>
     <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
     </dxf>
     <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
     </dxf>
     <dxf>
       <font>
@@ -1700,7 +1745,16 @@
       </font>
     </dxf>
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$€-40C]_-;\-* #,##0.00\ [$€-40C]_-;_-* &quot;-&quot;??\ [$€-40C]_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
     <dxf>
       <font>
@@ -1719,61 +1773,16 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
-      <numFmt numFmtId="0" formatCode="General"/>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$€-40C]_-;\-* #,##0.00\ [$€-40C]_-;_-* &quot;-&quot;??\ [$€-40C]_-;_-@_-"/>
     </dxf>
     <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1799,8 +1808,8 @@
     <tableColumn id="4" xr3:uid="{84F1F30D-4827-43F2-8865-B7957E3E712D}" name="ID"/>
     <tableColumn id="7" xr3:uid="{512EABBD-B863-4251-833D-8B8D1F1626EF}" name="Description"/>
     <tableColumn id="2" xr3:uid="{D09C4BB0-FEBD-4A72-9E87-B5258D8B62D7}" name="Label de la provision"/>
-    <tableColumn id="3" xr3:uid="{347751FB-EF14-4BD7-9D47-427E04136B77}" name="Provision" totalsRowFunction="sum" dataDxfId="25" totalsRowDxfId="24" dataCellStyle="Monétaire"/>
-    <tableColumn id="5" xr3:uid="{CA26B6F8-88AD-418A-B213-749ABA66E926}" name="Description longue" dataDxfId="23"/>
+    <tableColumn id="3" xr3:uid="{347751FB-EF14-4BD7-9D47-427E04136B77}" name="Provision" totalsRowFunction="sum" dataDxfId="22" totalsRowDxfId="21" dataCellStyle="Monétaire"/>
+    <tableColumn id="5" xr3:uid="{CA26B6F8-88AD-418A-B213-749ABA66E926}" name="Description longue" dataDxfId="20"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1813,47 +1822,47 @@
     <sortCondition ref="A1:A180"/>
   </sortState>
   <tableColumns count="16">
-    <tableColumn id="3" xr3:uid="{1687C042-C916-4161-82C2-2A915364FCD2}" name="Numéro de lot" dataDxfId="22"/>
+    <tableColumn id="3" xr3:uid="{1687C042-C916-4161-82C2-2A915364FCD2}" name="Numéro de lot" dataDxfId="19"/>
     <tableColumn id="1" xr3:uid="{788DBA8C-5B77-4079-8161-FA45C58518AE}" name="Description"/>
-    <tableColumn id="2" xr3:uid="{BE5ACA99-AEAF-4E51-BE0A-B3FB8FCCF08B}" name="Tantièmes copropriété" dataDxfId="21">
+    <tableColumn id="2" xr3:uid="{BE5ACA99-AEAF-4E51-BE0A-B3FB8FCCF08B}" name="Tantièmes copropriété" dataDxfId="18">
       <calculatedColumnFormula>7/10000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{D62FAA89-C46E-4AF6-A14F-7FD6F46E7F00}" name="Tantièmes ascenseur 1-1" dataDxfId="20"/>
-    <tableColumn id="9" xr3:uid="{C3B9BDED-CB2A-4305-9CBF-418F5971AC1E}" name="Tantièmes ascenseur 1-2" dataDxfId="19"/>
-    <tableColumn id="10" xr3:uid="{C2291DE1-C707-4F83-846E-F914B4B42E52}" name="Tantièmes ascenseur 2" dataDxfId="18"/>
-    <tableColumn id="11" xr3:uid="{4F70F08A-4C2F-41B0-88EB-711B1A0760CD}" name="Tantièmes ascenseur 3" dataDxfId="17"/>
-    <tableColumn id="14" xr3:uid="{80D23396-716C-46AC-9B55-BCBC6C981351}" name="Tantièmes chauffage" dataDxfId="16"/>
-    <tableColumn id="15" xr3:uid="{E3955139-B619-4DD0-8FC1-ECA97048DFE4}" name="Tantièmes Batiment 1" dataDxfId="15"/>
-    <tableColumn id="16" xr3:uid="{C73E9407-A858-4EF7-81C2-6C70C4B157A2}" name="Tantièmes Batiment 2" dataDxfId="14"/>
-    <tableColumn id="17" xr3:uid="{A07338CA-0096-4091-89B2-A46FF2D323C2}" name="Tantièmes Batiment 3" dataDxfId="13"/>
-    <tableColumn id="18" xr3:uid="{7A3012D8-2375-4F10-9E84-F2F5060C6A99}" name="Tantièmes Hall 1-1" dataDxfId="12"/>
-    <tableColumn id="19" xr3:uid="{67961B6E-B577-4A49-B099-623FB85519B4}" name="Tantièmes Hall 1-2" dataDxfId="11"/>
-    <tableColumn id="20" xr3:uid="{03C201C1-F8AA-4D3C-AEBC-425B180BC2D7}" name="Tantièmes Hall 2" dataDxfId="10"/>
-    <tableColumn id="21" xr3:uid="{4826FC05-81A9-4020-8D1D-83D3D5C5A05A}" name="Tantièmes Logement/Stationnements" dataDxfId="9"/>
-    <tableColumn id="6" xr3:uid="{7B87787E-3595-42D5-B815-AF76B67432D8}" name="Tantièmes Stationnement" dataDxfId="8"/>
+    <tableColumn id="8" xr3:uid="{D62FAA89-C46E-4AF6-A14F-7FD6F46E7F00}" name="Tantièmes ascenseur 1-1" dataDxfId="17"/>
+    <tableColumn id="9" xr3:uid="{C3B9BDED-CB2A-4305-9CBF-418F5971AC1E}" name="Tantièmes ascenseur 1-2" dataDxfId="16"/>
+    <tableColumn id="10" xr3:uid="{C2291DE1-C707-4F83-846E-F914B4B42E52}" name="Tantièmes ascenseur 2" dataDxfId="15"/>
+    <tableColumn id="11" xr3:uid="{4F70F08A-4C2F-41B0-88EB-711B1A0760CD}" name="Tantièmes ascenseur 3" dataDxfId="14"/>
+    <tableColumn id="14" xr3:uid="{80D23396-716C-46AC-9B55-BCBC6C981351}" name="Tantièmes chauffage" dataDxfId="13"/>
+    <tableColumn id="15" xr3:uid="{E3955139-B619-4DD0-8FC1-ECA97048DFE4}" name="Tantièmes Batiment 1" dataDxfId="12"/>
+    <tableColumn id="16" xr3:uid="{C73E9407-A858-4EF7-81C2-6C70C4B157A2}" name="Tantièmes Batiment 2" dataDxfId="11"/>
+    <tableColumn id="17" xr3:uid="{A07338CA-0096-4091-89B2-A46FF2D323C2}" name="Tantièmes Batiment 3" dataDxfId="10"/>
+    <tableColumn id="18" xr3:uid="{7A3012D8-2375-4F10-9E84-F2F5060C6A99}" name="Tantièmes Hall 1-1" dataDxfId="9"/>
+    <tableColumn id="19" xr3:uid="{67961B6E-B577-4A49-B099-623FB85519B4}" name="Tantièmes Hall 1-2" dataDxfId="8"/>
+    <tableColumn id="20" xr3:uid="{03C201C1-F8AA-4D3C-AEBC-425B180BC2D7}" name="Tantièmes Hall 2" dataDxfId="7"/>
+    <tableColumn id="21" xr3:uid="{4826FC05-81A9-4020-8D1D-83D3D5C5A05A}" name="Tantièmes Logement/Stationnements" dataDxfId="6"/>
+    <tableColumn id="6" xr3:uid="{7B87787E-3595-42D5-B815-AF76B67432D8}" name="Tantièmes Stationnement" dataDxfId="5"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{AFF80A4D-E18B-42B5-9271-DD654E188D32}" name="Prestations" displayName="Prestations" ref="A1:I37" totalsRowShown="0">
-  <autoFilter ref="A1:I37" xr:uid="{AFF80A4D-E18B-42B5-9271-DD654E188D32}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{AFF80A4D-E18B-42B5-9271-DD654E188D32}" name="Prestations" displayName="Prestations" ref="A1:I38" totalsRowShown="0">
+  <autoFilter ref="A1:I38" xr:uid="{AFF80A4D-E18B-42B5-9271-DD654E188D32}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H37">
     <sortCondition ref="B1:B37"/>
   </sortState>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{7753A616-C6B5-4B02-AE3F-2A95253630B8}" name="Type de prestation" dataDxfId="7"/>
-    <tableColumn id="2" xr3:uid="{D7B6EA29-CA0A-4C24-9A81-3DF01785BD0C}" name="Label de la prestation" dataDxfId="6"/>
-    <tableColumn id="8" xr3:uid="{91FE62B8-BF79-4277-91C2-4B3C13901105}" name="ID prestation" dataDxfId="5"/>
+    <tableColumn id="1" xr3:uid="{7753A616-C6B5-4B02-AE3F-2A95253630B8}" name="Type de prestation" dataDxfId="30"/>
+    <tableColumn id="2" xr3:uid="{D7B6EA29-CA0A-4C24-9A81-3DF01785BD0C}" name="Label de la prestation" dataDxfId="29"/>
+    <tableColumn id="8" xr3:uid="{91FE62B8-BF79-4277-91C2-4B3C13901105}" name="ID prestation" dataDxfId="28"/>
     <tableColumn id="3" xr3:uid="{2ADF6FF1-1416-43FA-A9BF-E696654CC8CD}" name="Prestataire"/>
-    <tableColumn id="4" xr3:uid="{1C295B62-0191-41FA-9660-5BADE532BEE7}" name="Cout" dataDxfId="4"/>
-    <tableColumn id="5" xr3:uid="{1E3C456B-12BB-4B06-B366-57CE3DA87819}" name="Taxes" dataDxfId="3"/>
-    <tableColumn id="6" xr3:uid="{20997A37-E6E3-4308-9ACD-8D77B289D813}" name="Total TTC" dataDxfId="2">
+    <tableColumn id="4" xr3:uid="{1C295B62-0191-41FA-9660-5BADE532BEE7}" name="Cout" dataDxfId="27"/>
+    <tableColumn id="5" xr3:uid="{1E3C456B-12BB-4B06-B366-57CE3DA87819}" name="Taxes" dataDxfId="26"/>
+    <tableColumn id="6" xr3:uid="{20997A37-E6E3-4308-9ACD-8D77B289D813}" name="Total TTC" dataDxfId="25">
       <calculatedColumnFormula>IF(Prestations[[#This Row],[Taxes]]="TTC",Prestations[[#This Row],[Cout]],Prestations[[#This Row],[Cout]]*1.2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{6BDB0ED6-23A7-4E1A-A654-9E18B0DA38B5}" name="Description" dataDxfId="1"/>
-    <tableColumn id="9" xr3:uid="{C919E254-DE7F-4D3B-8CF6-79E643BBF97F}" name="Prestation choisie actuellement" dataDxfId="0"/>
+    <tableColumn id="7" xr3:uid="{6BDB0ED6-23A7-4E1A-A654-9E18B0DA38B5}" name="Description" dataDxfId="24"/>
+    <tableColumn id="9" xr3:uid="{C919E254-DE7F-4D3B-8CF6-79E643BBF97F}" name="Prestation choisie actuellement" dataDxfId="23"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1880,13 +1889,13 @@
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{455C30A6-2C19-4BD7-B8A4-D1C6252917DD}" name="Type de chaudière"/>
     <tableColumn id="2" xr3:uid="{FAAC8507-DC80-422C-8508-496178C23374}" name="ID poste de provision"/>
-    <tableColumn id="3" xr3:uid="{17764D71-05D7-4B37-8536-4004CBBE2CD4}" name="Prix unitaire du kWh" dataDxfId="30"/>
-    <tableColumn id="7" xr3:uid="{39B6FB9A-9DCB-412D-8CBD-94E321E39A50}" name="Unité" dataDxfId="29"/>
-    <tableColumn id="8" xr3:uid="{C769AD0E-5A43-462D-8737-CE59FA9E9F57}" name="Prix TTC de l'unité" dataDxfId="28"/>
-    <tableColumn id="9" xr3:uid="{C32F2A17-C994-4DCC-A33C-2604586EDB4F}" name="kWh par unité" dataDxfId="27"/>
+    <tableColumn id="3" xr3:uid="{17764D71-05D7-4B37-8536-4004CBBE2CD4}" name="Prix unitaire du kWh" dataDxfId="4"/>
+    <tableColumn id="7" xr3:uid="{39B6FB9A-9DCB-412D-8CBD-94E321E39A50}" name="Unité" dataDxfId="3"/>
+    <tableColumn id="8" xr3:uid="{C769AD0E-5A43-462D-8737-CE59FA9E9F57}" name="Prix TTC de l'unité" dataDxfId="2"/>
+    <tableColumn id="9" xr3:uid="{C32F2A17-C994-4DCC-A33C-2604586EDB4F}" name="kWh par unité" dataDxfId="1"/>
     <tableColumn id="4" xr3:uid="{FECEDA0B-3F17-4D04-AB3F-B1B848AA5DB2}" name="Production maximum en kW"/>
     <tableColumn id="6" xr3:uid="{F8EB0843-7F05-427F-9B41-0852730F32C9}" name="Description"/>
-    <tableColumn id="10" xr3:uid="{9F9F9E98-6D66-4867-A354-22539BFC6A70}" name="Seuil de fonctionnement (kW)" dataDxfId="26"/>
+    <tableColumn id="10" xr3:uid="{9F9F9E98-6D66-4867-A354-22539BFC6A70}" name="Seuil de fonctionnement (kW)" dataDxfId="0"/>
     <tableColumn id="11" xr3:uid="{D0B5F61C-1D85-4C5E-A117-B774F88FE50E}" name="Seuil de durée d'activation (mn)"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -6880,7 +6889,7 @@
   <sheetPr>
     <tabColor theme="9" tint="0.79998168889431442"/>
   </sheetPr>
-  <dimension ref="A1:I37"/>
+  <dimension ref="A1:I38"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="48.140625" customWidth="1"/>
@@ -7873,6 +7882,33 @@
       </c>
       <c r="I37" s="2" t="s">
         <v>188</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A38" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>405</v>
+      </c>
+      <c r="C38" t="s">
+        <v>72</v>
+      </c>
+      <c r="D38" t="s">
+        <v>406</v>
+      </c>
+      <c r="E38" s="4">
+        <v>10932.1</v>
+      </c>
+      <c r="F38" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="G38" s="4">
+        <f>IF(Prestations[[#This Row],[Taxes]]="TTC",Prestations[[#This Row],[Cout]],Prestations[[#This Row],[Cout]]*1.2)</f>
+        <v>13118.52</v>
+      </c>
+      <c r="H38" s="2" t="s">
+        <v>407</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Mis à jour prix combustible
</commit_message>
<xml_diff>
--- a/input.xlsx
+++ b/input.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/25a393584c41f6f2/Documents/Mon Patrimoine/Projet Immobilier/2023 Terrasses de Galieni/09 - Copropriété/Site de calcul des charges de copropriété/streamlit-copro-charges/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1366" documentId="13_ncr:1_{471232EB-3AAB-4D08-BC1C-7B7CD1C1D853}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{75ADD3F5-8AE0-40BD-9CA2-45A4CD25B930}"/>
+  <xr:revisionPtr revIDLastSave="1367" documentId="13_ncr:1_{471232EB-3AAB-4D08-BC1C-7B7CD1C1D853}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2F4AC2A7-AD15-4D68-8B7A-52210FB393DD}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Provisions" sheetId="9" r:id="rId1"/>
@@ -8052,8 +8052,8 @@
         <v>397</v>
       </c>
       <c r="E2" s="1">
-        <f>392*1.2</f>
-        <v>470.4</v>
+        <f>310*1.2</f>
+        <v>372</v>
       </c>
       <c r="F2" s="12">
         <v>4900</v>

</xml_diff>

<commit_message>
MAJ paramètre par défaut et VMC
</commit_message>
<xml_diff>
--- a/input.xlsx
+++ b/input.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/25a393584c41f6f2/Documents/Mon Patrimoine/Projet Immobilier/2023 Terrasses de Galieni/09 - Copropriété/Site de calcul des charges de copropriété/streamlit-copro-charges/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1367" documentId="13_ncr:1_{471232EB-3AAB-4D08-BC1C-7B7CD1C1D853}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2F4AC2A7-AD15-4D68-8B7A-52210FB393DD}"/>
+  <xr:revisionPtr revIDLastSave="1419" documentId="13_ncr:1_{471232EB-3AAB-4D08-BC1C-7B7CD1C1D853}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EE078EAE-918E-4E5C-9DF0-DB525F631E88}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Provisions" sheetId="9" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="600" uniqueCount="408">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="626" uniqueCount="417">
   <si>
     <t>Taxes</t>
   </si>
@@ -1277,6 +1277,42 @@
   </si>
   <si>
     <t>Contrat P2, engagement sur 3 ans, a priori pas de livraison</t>
+  </si>
+  <si>
+    <t>Consommation de sel pour adoucir l'eau - Estimation basse</t>
+  </si>
+  <si>
+    <t>Esimation IA</t>
+  </si>
+  <si>
+    <t>L’adoucisseur est récent et volumétrique : il se régénère selon le volume d’eau réellement consommé, et non selon un calendrier fixe.
+La régénération se fait à contre-courant, ce qui économise du sel.
+Le réglage est bien ajusté, avec un mitigeur de dureté qui laisse passer une partie d’eau brute.
+Il consomme 25 g de sel par °f·m³, soit 0,8 t par an.
+Le sel est acheté au prix du détail le plus bas, 0,40 €/kg (pastilles en sac de 25 kg), ce qui donne environ 320 €.</t>
+  </si>
+  <si>
+    <t>L’appareil est fonctionnel mais pas optimisé : réglage standard du fabricant, régénération moins économe.
+Il consomme 40 g par °f·m³, soit 1,3 t par an.
+Le sel coûte 0,50 €/kg, par exemple en achat groupé ou livré, ce qui donne environ 640 €.
+C’est ce que je considère comme le cas le plus probable pour une résidence sans suivi particulier.</t>
+  </si>
+  <si>
+    <t>L’appareil est ancien, régénéré au chronomètre, c’est-à-dire à intervalles fixes même si l’eau n’a pas été consommée, ou surdimensionné. Il peut aussi être réglé pour descendre trop bas en dureté.
+Il consomme 80 g par °f·m³, soit 2,6 t par an.
+Le sel coûte 0,70 €/kg, avec livraison et petites quantités, ce qui donne environ 1 800 €.</t>
+  </si>
+  <si>
+    <t>Maintenance de la VMC</t>
+  </si>
+  <si>
+    <t>Consommation de sel pour adoucir l'eau</t>
+  </si>
+  <si>
+    <t>Inclus dans le contrat P2 de Dalkia (pas de prix exact)</t>
+  </si>
+  <si>
+    <t>Maintenance de la VMC Dalkia</t>
   </si>
 </sst>
 </file>
@@ -1323,7 +1359,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -1342,13 +1378,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1368,6 +1413,9 @@
     <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Monétaire" xfId="1" builtinId="4"/>
@@ -1846,8 +1894,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{AFF80A4D-E18B-42B5-9271-DD654E188D32}" name="Prestations" displayName="Prestations" ref="A1:I38" totalsRowShown="0">
-  <autoFilter ref="A1:I38" xr:uid="{AFF80A4D-E18B-42B5-9271-DD654E188D32}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{AFF80A4D-E18B-42B5-9271-DD654E188D32}" name="Prestations" displayName="Prestations" ref="A1:I42" totalsRowShown="0">
+  <autoFilter ref="A1:I42" xr:uid="{AFF80A4D-E18B-42B5-9271-DD654E188D32}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H37">
     <sortCondition ref="B1:B37"/>
   </sortState>
@@ -6889,17 +6937,17 @@
   <sheetPr>
     <tabColor theme="9" tint="0.79998168889431442"/>
   </sheetPr>
-  <dimension ref="A1:I38"/>
+  <dimension ref="A1:I43"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="48.140625" customWidth="1"/>
+    <col min="1" max="1" width="47.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="66.5703125" style="2" customWidth="1"/>
     <col min="3" max="3" width="15.5703125" style="2" customWidth="1"/>
     <col min="4" max="4" width="32.85546875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11.85546875" style="4" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="8.28515625" style="6" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="12.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="124.7109375" style="2" customWidth="1"/>
+    <col min="8" max="8" width="132.5703125" style="2" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="31.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -7913,6 +7961,128 @@
       <c r="I38" t="s">
         <v>188</v>
       </c>
+    </row>
+    <row r="39" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+      <c r="A39" s="2" t="s">
+        <v>414</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="C39" t="s">
+        <v>72</v>
+      </c>
+      <c r="D39" t="s">
+        <v>409</v>
+      </c>
+      <c r="E39" s="4">
+        <v>320</v>
+      </c>
+      <c r="F39" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="G39" s="4">
+        <f>IF(Prestations[[#This Row],[Taxes]]="TTC",Prestations[[#This Row],[Cout]],Prestations[[#This Row],[Cout]]*1.2)</f>
+        <v>320</v>
+      </c>
+      <c r="H39" s="2" t="s">
+        <v>410</v>
+      </c>
+      <c r="I39" s="2"/>
+    </row>
+    <row r="40" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+      <c r="A40" s="2" t="s">
+        <v>414</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="C40" t="s">
+        <v>72</v>
+      </c>
+      <c r="D40" t="s">
+        <v>409</v>
+      </c>
+      <c r="E40" s="4">
+        <v>640</v>
+      </c>
+      <c r="F40" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="G40" s="13">
+        <f>IF(Prestations[[#This Row],[Taxes]]="TTC",Prestations[[#This Row],[Cout]],Prestations[[#This Row],[Cout]]*1.2)</f>
+        <v>640</v>
+      </c>
+      <c r="H40" s="2" t="s">
+        <v>411</v>
+      </c>
+      <c r="I40" s="2" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+      <c r="A41" s="2" t="s">
+        <v>414</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="D41" t="s">
+        <v>409</v>
+      </c>
+      <c r="E41" s="14">
+        <v>1800</v>
+      </c>
+      <c r="F41" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="G41" s="15">
+        <f>IF(Prestations[[#This Row],[Taxes]]="TTC",Prestations[[#This Row],[Cout]],Prestations[[#This Row],[Cout]]*1.2)</f>
+        <v>1800</v>
+      </c>
+      <c r="H41" s="2" t="s">
+        <v>412</v>
+      </c>
+      <c r="I41" s="2"/>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>413</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>416</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="D42" t="s">
+        <v>406</v>
+      </c>
+      <c r="E42" s="4">
+        <v>0</v>
+      </c>
+      <c r="F42" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="G42" s="15">
+        <f>IF(Prestations[[#This Row],[Taxes]]="TTC",Prestations[[#This Row],[Cout]],Prestations[[#This Row],[Cout]]*1.2)</f>
+        <v>0</v>
+      </c>
+      <c r="H42" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="I42" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A43" s="2"/>
+      <c r="C43"/>
+      <c r="G43" s="13"/>
+      <c r="I43" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -7926,7 +8096,7 @@
           <x14:formula1>
             <xm:f>Provisions!$B:$B</xm:f>
           </x14:formula1>
-          <xm:sqref>C1:C1048576</xm:sqref>
+          <xm:sqref>C45:C1048576 C1:C43</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>

<commit_message>
MAJ si prestata selectionnee alors on prends ça plutôt que prov
</commit_message>
<xml_diff>
--- a/input.xlsx
+++ b/input.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/25a393584c41f6f2/Documents/Mon Patrimoine/Projet Immobilier/2023 Terrasses de Galieni/09 - Copropriété/Site de calcul des charges de copropriété/streamlit-copro-charges/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1419" documentId="13_ncr:1_{471232EB-3AAB-4D08-BC1C-7B7CD1C1D853}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EE078EAE-918E-4E5C-9DF0-DB525F631E88}"/>
+  <xr:revisionPtr revIDLastSave="1421" documentId="13_ncr:1_{471232EB-3AAB-4D08-BC1C-7B7CD1C1D853}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5433CA94-0E5A-44AE-8A12-0AC1B99ADD97}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="626" uniqueCount="417">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="626" uniqueCount="419">
   <si>
     <t>Taxes</t>
   </si>
@@ -1313,6 +1313,12 @@
   </si>
   <si>
     <t>Maintenance de la VMC Dalkia</t>
+  </si>
+  <si>
+    <t>Consommation de sel pour adoucir l'eau - Estimation moyenne</t>
+  </si>
+  <si>
+    <t>Consommation de sel pour adoucir l'eau - Estimation haute</t>
   </si>
 </sst>
 </file>
@@ -7995,7 +8001,7 @@
         <v>414</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>408</v>
+        <v>417</v>
       </c>
       <c r="C40" t="s">
         <v>72</v>
@@ -8025,7 +8031,7 @@
         <v>414</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>408</v>
+        <v>418</v>
       </c>
       <c r="C41" s="2" t="s">
         <v>72</v>

</xml_diff>